<commit_message>
app for final demo version done
</commit_message>
<xml_diff>
--- a/Updated Data Pull Example.xlsx
+++ b/Updated Data Pull Example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wenxi/school/nu/NPS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BDA9FDB8-CBDC-4342-8B64-4ABC38DCB1C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5CBAC21-3EDE-FF46-900B-70A0215DC02F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14580" yWindow="-20980" windowWidth="19200" windowHeight="20980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="21660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Contact Reports in the last 60 " sheetId="1" r:id="rId1"/>
@@ -268,7 +268,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -294,6 +294,7 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -628,7 +629,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X3"/>
+  <dimension ref="A1:X4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
@@ -879,6 +880,10 @@
         <v>44</v>
       </c>
     </row>
+    <row r="4" spans="1:24" ht="16" x14ac:dyDescent="0.2">
+      <c r="A4" s="2"/>
+      <c r="B4" s="13"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>